<commit_message>
Better one-to-one checks and representation
</commit_message>
<xml_diff>
--- a/inst/rules/qc_rules.xlsx
+++ b/inst/rules/qc_rules.xlsx
@@ -8533,7 +8533,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>scientificName and scientificNameID do not go one-to-one</t>
+          <t>Broken one-to-one: scientificName and scientificNameID</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -8608,7 +8608,7 @@
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>One value with several IDs is reported with the check's severity; one ID with several values (usually spelling) as warning.</t>
+          <t>Both ways are errors: a value with several IDs, and an ID with several values. Every combination is listed next to each other on the Overview (Values and their IDs), on screen 3 when the problem is chosen, and by qc_one_to_one(). A name without ID (or an ID without name) while other records have one: warning.</t>
         </is>
       </c>
     </row>
@@ -9361,12 +9361,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Value and value ID do not go one-to-one</t>
+          <t>Broken one-to-one: measurementValue and measurementValueID</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>error</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -9436,7 +9436,7 @@
       </c>
       <c r="R95" t="inlineStr">
         <is>
-          <t/>
+          <t>Both ways are errors: a value with several IDs, and an ID with several values. Every combination is listed next to each other on the Overview (Values and their IDs), on screen 3 when the problem is chosen, and by qc_one_to_one(). Text values are compared within each measurement type. A text value without valueID while other records of it have one: warning.</t>
         </is>
       </c>
     </row>
@@ -9453,7 +9453,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>measurementType and measurementTypeID do not go one-to-one</t>
+          <t>Broken one-to-one: measurementType and measurementTypeID</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -9528,7 +9528,7 @@
       </c>
       <c r="R96" t="inlineStr">
         <is>
-          <t>One value with several IDs is reported with the check's severity; one ID with several values (usually spelling) as warning.</t>
+          <t>Both ways are errors: a value with several IDs, and an ID with several values. Every combination is listed next to each other on the Overview (Values and their IDs), on screen 3 when the problem is chosen, and by qc_one_to_one().</t>
         </is>
       </c>
     </row>
@@ -9545,7 +9545,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>measurementUnit and measurementUnitID do not go one-to-one</t>
+          <t>Broken one-to-one: measurementUnit and measurementUnitID</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -9620,7 +9620,7 @@
       </c>
       <c r="R97" t="inlineStr">
         <is>
-          <t>One value with several IDs is reported with the check's severity; one ID with several values (usually spelling) as warning.</t>
+          <t>Both ways are errors: a value with several IDs, and an ID with several values. Every combination is listed next to each other on the Overview (Values and their IDs), on screen 3 when the problem is chosen, and by qc_one_to_one().</t>
         </is>
       </c>
     </row>
@@ -12029,12 +12029,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Other values and their IDs do not go one-to-one</t>
+          <t>Broken one-to-one: other values and their IDs</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>error</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -12104,7 +12104,7 @@
       </c>
       <c r="R124" t="inlineStr">
         <is>
-          <t>The DM team can add pairs to the list.</t>
+          <t>Both ways are errors: a value with several IDs, and an ID with several values. Every combination is listed next to each other on the Overview (Values and their IDs), on screen 3 when the problem is chosen, and by qc_one_to_one(). The DM team can add pairs to the list.</t>
         </is>
       </c>
     </row>

</xml_diff>